<commit_message>
fix:email to multiple person
</commit_message>
<xml_diff>
--- a/media/demo_files/demo_calendar.xlsx
+++ b/media/demo_files/demo_calendar.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -476,7 +476,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -496,7 +496,7 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -516,7 +516,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -536,7 +536,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Added topic edit & delete
</commit_message>
<xml_diff>
--- a/media/demo_files/demo_calendar.xlsx
+++ b/media/demo_files/demo_calendar.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46186</v>
+        <v>46190</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -465,7 +465,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Text Post</t>
+          <t>Carousel</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -476,7 +476,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46187</v>
+        <v>46191</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -485,7 +485,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Reel</t>
+          <t>Carousel</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -496,7 +496,7 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46188</v>
+        <v>46192</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -516,7 +516,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46189</v>
+        <v>46193</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -536,7 +536,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46190</v>
+        <v>46194</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>

</xml_diff>